<commit_message>
POINT BASED SAFER DRAFT WAS FINISHED!
</commit_message>
<xml_diff>
--- a/Examples/samples.xlsx
+++ b/Examples/samples.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\pySAFER\Examples\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2542AC6D-CB83-4818-99A4-5034D8898875}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57F0B030-F06A-4B24-8F0A-D451AEF63319}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="40850" yWindow="2240" windowWidth="12220" windowHeight="18700" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>lat</t>
   </si>
@@ -63,6 +63,9 @@
   </si>
   <si>
     <t>eto</t>
+  </si>
+  <si>
+    <t>elevation</t>
   </si>
 </sst>
 </file>
@@ -380,10 +383,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I37"/>
+  <dimension ref="A1:J37"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -411,8 +414,11 @@
       <c r="I1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>20250501</v>
       </c>
@@ -440,8 +446,11 @@
       <c r="I2">
         <v>10</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J2">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>20250502</v>
       </c>
@@ -469,8 +478,11 @@
       <c r="I3">
         <v>10</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J3">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>20250503</v>
       </c>
@@ -498,8 +510,11 @@
       <c r="I4">
         <v>10</v>
       </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J4">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>20250504</v>
       </c>
@@ -527,8 +542,11 @@
       <c r="I5">
         <v>10</v>
       </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J5">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>20250505</v>
       </c>
@@ -556,8 +574,11 @@
       <c r="I6">
         <v>10</v>
       </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J6">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>20250506</v>
       </c>
@@ -585,8 +606,11 @@
       <c r="I7">
         <v>10</v>
       </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J7">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>20250507</v>
       </c>
@@ -614,8 +638,11 @@
       <c r="I8">
         <v>10</v>
       </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J8">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>20250508</v>
       </c>
@@ -643,8 +670,11 @@
       <c r="I9">
         <v>10</v>
       </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J9">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>20250509</v>
       </c>
@@ -672,8 +702,11 @@
       <c r="I10">
         <v>10</v>
       </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J10">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>20250510</v>
       </c>
@@ -701,8 +734,11 @@
       <c r="I11">
         <v>10</v>
       </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J11">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>20250511</v>
       </c>
@@ -730,8 +766,11 @@
       <c r="I12">
         <v>10</v>
       </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J12">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>20250512</v>
       </c>
@@ -759,8 +798,11 @@
       <c r="I13">
         <v>10</v>
       </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J13">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>20250513</v>
       </c>
@@ -788,8 +830,11 @@
       <c r="I14">
         <v>10</v>
       </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J14">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>20250514</v>
       </c>
@@ -817,8 +862,11 @@
       <c r="I15">
         <v>10</v>
       </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J15">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>20250515</v>
       </c>
@@ -846,8 +894,11 @@
       <c r="I16">
         <v>10</v>
       </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J16">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>20250516</v>
       </c>
@@ -875,8 +926,11 @@
       <c r="I17">
         <v>10</v>
       </c>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J17">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>20250517</v>
       </c>
@@ -904,8 +958,11 @@
       <c r="I18">
         <v>10</v>
       </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J18">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>20250518</v>
       </c>
@@ -933,8 +990,11 @@
       <c r="I19">
         <v>10</v>
       </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J19">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>20250519</v>
       </c>
@@ -962,8 +1022,11 @@
       <c r="I20">
         <v>10</v>
       </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J20">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>20250520</v>
       </c>
@@ -991,8 +1054,11 @@
       <c r="I21">
         <v>10</v>
       </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J21">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>20250521</v>
       </c>
@@ -1020,8 +1086,11 @@
       <c r="I22">
         <v>10</v>
       </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J22">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>20250522</v>
       </c>
@@ -1049,8 +1118,11 @@
       <c r="I23">
         <v>10</v>
       </c>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J23">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>20250523</v>
       </c>
@@ -1078,8 +1150,11 @@
       <c r="I24">
         <v>10</v>
       </c>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J24">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>20250524</v>
       </c>
@@ -1107,8 +1182,11 @@
       <c r="I25">
         <v>10</v>
       </c>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J25">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>20250525</v>
       </c>
@@ -1136,8 +1214,11 @@
       <c r="I26">
         <v>10</v>
       </c>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J26">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>20250526</v>
       </c>
@@ -1165,8 +1246,11 @@
       <c r="I27">
         <v>10</v>
       </c>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J27">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>20250527</v>
       </c>
@@ -1194,8 +1278,11 @@
       <c r="I28">
         <v>10</v>
       </c>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J28">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>20250528</v>
       </c>
@@ -1223,8 +1310,11 @@
       <c r="I29">
         <v>10</v>
       </c>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J29">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>20250529</v>
       </c>
@@ -1252,8 +1342,11 @@
       <c r="I30">
         <v>10</v>
       </c>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J30">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A31">
         <v>20250530</v>
       </c>
@@ -1281,8 +1374,11 @@
       <c r="I31">
         <v>10</v>
       </c>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J31">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A32">
         <v>20250531</v>
       </c>
@@ -1310,8 +1406,11 @@
       <c r="I32">
         <v>10</v>
       </c>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J32">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A33">
         <v>20250601</v>
       </c>
@@ -1339,8 +1438,11 @@
       <c r="I33">
         <v>12</v>
       </c>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J33">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A34">
         <v>20250602</v>
       </c>
@@ -1368,8 +1470,11 @@
       <c r="I34">
         <v>12</v>
       </c>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J34">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A35">
         <v>20250603</v>
       </c>
@@ -1397,8 +1502,11 @@
       <c r="I35">
         <v>12</v>
       </c>
-    </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J35">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A36">
         <v>20250604</v>
       </c>
@@ -1426,8 +1534,11 @@
       <c r="I36">
         <v>12</v>
       </c>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J36">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A37">
         <v>20250605</v>
       </c>
@@ -1454,6 +1565,9 @@
       </c>
       <c r="I37">
         <v>12</v>
+      </c>
+      <c r="J37">
+        <v>65</v>
       </c>
     </row>
   </sheetData>

</xml_diff>